<commit_message>
Updated the profit calc engine
</commit_message>
<xml_diff>
--- a/History_for_Account_Z33464548.xlsx
+++ b/History_for_Account_Z33464548.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a7d5810855f5c874/Documents/Investments/US Index Investments/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a7d5810855f5c874/Documents/Investments/USindextracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{68E739DE-E969-426F-968E-38023C5E8ECE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A283D817-AD43-40BA-B8DC-FD579FB493CE}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{68E739DE-E969-426F-968E-38023C5E8ECE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9DF813DF-1B14-4F7E-B15B-A1C43E16C288}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{3309808E-588E-4831-9D85-3065AC75138B}"/>
   </bookViews>
@@ -807,10 +807,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1132,6 +1128,7 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="109.36328125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="34.90625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="14.08984375" bestFit="1" customWidth="1"/>
   </cols>

</xml_diff>